<commit_message>
influencer CRM: add Hayley Carter (@hayley__carter) prospect
72.3k Dallas motherhood/lifestyle creator, agency-repped (It Girl Agency).
Lane A, provisional rating 4 pending media-kit engagement + audience US-geo.

Co-Authored-By: Claude Opus 4.7 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/marketing/influencer/influencer-crm.xlsx
+++ b/marketing/influencer/influencer-crm.xlsx
@@ -11,7 +11,7 @@
     <sheet name="Rubric &amp; Legend" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Influencer CRM'!$A$1:$N$18</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Influencer CRM'!$A$1:$N$19</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="0">'Influencer CRM'!$1:$1</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -521,7 +521,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:N18"/>
+  <dimension ref="A1:N19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -1175,55 +1175,55 @@
     <row r="10">
       <c r="A10" s="11" t="inlineStr">
         <is>
-          <t>Kristen Corrao</t>
+          <t>Hayley Carter</t>
         </is>
       </c>
       <c r="B10" s="11" t="inlineStr">
         <is>
-          <t>@kristen_corrao</t>
+          <t>@hayley__carter</t>
         </is>
       </c>
       <c r="C10" s="12" t="inlineStr">
         <is>
-          <t>IG / TikTok</t>
+          <t>IG</t>
         </is>
       </c>
       <c r="D10" s="12" t="inlineStr">
         <is>
-          <t>1.2k IG / 22.8k TT</t>
+          <t>72.3k</t>
         </is>
       </c>
       <c r="E10" s="11" t="inlineStr">
         <is>
-          <t>Collabstr (parenting)</t>
+          <t>Dan-sourced / IG direct</t>
         </is>
       </c>
       <c r="F10" s="11" t="inlineStr">
         <is>
-          <t>Motherhood / parenting</t>
+          <t>Motherhood / lifestyle / wellness; mom of 4; Dallas TX</t>
         </is>
       </c>
       <c r="G10" s="12" t="inlineStr">
         <is>
-          <t>88%</t>
+          <t>unknown (she's US)</t>
         </is>
       </c>
       <c r="H10" s="12" t="inlineStr">
         <is>
-          <t>18.7%</t>
+          <t>unknown</t>
         </is>
       </c>
       <c r="I10" s="11" t="inlineStr">
         <is>
-          <t>$70 feed</t>
+          <t>unknown (agency-quoted)</t>
         </is>
       </c>
       <c r="J10" s="13" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="K10" s="12" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>A</t>
         </is>
       </c>
       <c r="L10" s="12" t="inlineStr">
@@ -1233,34 +1233,34 @@
       </c>
       <c r="M10" s="12" t="inlineStr">
         <is>
-          <t>2026-06-10 (researched)</t>
+          <t>—</t>
         </is>
       </c>
       <c r="N10" s="11" t="inlineStr">
         <is>
-          <t>Excellent: 88% US, 71% F, 74% target age, Top Creator. Tiny IG following -&gt; Lane B: recurring affiliate (35%) likely beats one-shot paid. If paid: cheapest high-fit option at $70.</t>
+          <t>PROVISIONAL rating 4 — strong on visible signals (US-based Dallas creator, motherhood niche, public 'Digital creator', healthy 72k/1.7k follow ratio) but engagement % and audience US-geo are UNVERIFIED. AGENCY-REPPED: outreach goes to teamhayley@itgirlagency.com (email is the front door, not a cold DM). Bio: 'faith family fitness fashion, relatable mom content + wellness + ootd.' linktr.ee/HayleyCarter. Ask the agency for a media kit (engagement + audience geography) BEFORE committing budget; wants a permanent feed post (stays on grid).</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="11" t="inlineStr">
         <is>
-          <t>Jennifer Mendez</t>
+          <t>Kristen Corrao</t>
         </is>
       </c>
       <c r="B11" s="11" t="inlineStr">
         <is>
-          <t>@jenn11</t>
+          <t>@kristen_corrao</t>
         </is>
       </c>
       <c r="C11" s="12" t="inlineStr">
         <is>
-          <t>IG</t>
+          <t>IG / TikTok</t>
         </is>
       </c>
       <c r="D11" s="12" t="inlineStr">
         <is>
-          <t>2.2k</t>
+          <t>1.2k IG / 22.8k TT</t>
         </is>
       </c>
       <c r="E11" s="11" t="inlineStr">
@@ -1270,26 +1270,26 @@
       </c>
       <c r="F11" s="11" t="inlineStr">
         <is>
-          <t>Lifestyle / parenting</t>
+          <t>Motherhood / parenting</t>
         </is>
       </c>
       <c r="G11" s="12" t="inlineStr">
         <is>
-          <t>98%</t>
+          <t>88%</t>
         </is>
       </c>
       <c r="H11" s="12" t="inlineStr">
         <is>
-          <t>2.0%</t>
+          <t>18.7%</t>
         </is>
       </c>
       <c r="I11" s="11" t="inlineStr">
         <is>
-          <t>$85 feed</t>
+          <t>$70 feed</t>
         </is>
       </c>
       <c r="J11" s="13" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="K11" s="12" t="inlineStr">
         <is>
@@ -1308,54 +1308,54 @@
       </c>
       <c r="N11" s="11" t="inlineStr">
         <is>
-          <t>Highest US% of anyone (98%); 117k avg views (punches above follower count). 55% F (lower than ideal), age 25-34 52%. Fort Worth TX, 5.0 rating. Tiny following -&gt; Lane B affiliate-first.</t>
+          <t>Excellent: 88% US, 71% F, 74% target age, Top Creator. Tiny IG following -&gt; Lane B: recurring affiliate (35%) likely beats one-shot paid. If paid: cheapest high-fit option at $70.</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="11" t="inlineStr">
         <is>
-          <t>Denise Ferreira</t>
+          <t>Jennifer Mendez</t>
         </is>
       </c>
       <c r="B12" s="11" t="inlineStr">
         <is>
-          <t>@deniiseferreira</t>
+          <t>@jenn11</t>
         </is>
       </c>
       <c r="C12" s="12" t="inlineStr">
         <is>
-          <t>IG / TikTok</t>
+          <t>IG</t>
         </is>
       </c>
       <c r="D12" s="12" t="inlineStr">
         <is>
-          <t>12.4k</t>
+          <t>2.2k</t>
         </is>
       </c>
       <c r="E12" s="11" t="inlineStr">
         <is>
-          <t>Collabstr (mommy)</t>
+          <t>Collabstr (parenting)</t>
         </is>
       </c>
       <c r="F12" s="11" t="inlineStr">
         <is>
-          <t>Mommy / lifestyle</t>
+          <t>Lifestyle / parenting</t>
         </is>
       </c>
       <c r="G12" s="12" t="inlineStr">
         <is>
-          <t>85%</t>
+          <t>98%</t>
         </is>
       </c>
       <c r="H12" s="12" t="inlineStr">
         <is>
-          <t>0.4% IG</t>
+          <t>2.0%</t>
         </is>
       </c>
       <c r="I12" s="11" t="inlineStr">
         <is>
-          <t>$100 feed</t>
+          <t>$85 feed</t>
         </is>
       </c>
       <c r="J12" s="13" t="n">
@@ -1363,7 +1363,7 @@
       </c>
       <c r="K12" s="12" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>B</t>
         </is>
       </c>
       <c r="L12" s="12" t="inlineStr">
@@ -1378,39 +1378,39 @@
       </c>
       <c r="N12" s="11" t="inlineStr">
         <is>
-          <t>85% US, 96% F (highest), 68% target age. IG engagement low (0.4%) but TikTok viral (318k avg views). San Diego CA. Strong demo; value buy.</t>
+          <t>Highest US% of anyone (98%); 117k avg views (punches above follower count). 55% F (lower than ideal), age 25-34 52%. Fort Worth TX, 5.0 rating. Tiny following -&gt; Lane B affiliate-first.</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="11" t="inlineStr">
         <is>
-          <t>Alexandra 'Jax' Molieri</t>
+          <t>Denise Ferreira</t>
         </is>
       </c>
       <c r="B13" s="11" t="inlineStr">
         <is>
-          <t>@jaxdisneyfam</t>
+          <t>@deniiseferreira</t>
         </is>
       </c>
       <c r="C13" s="12" t="inlineStr">
         <is>
-          <t>IG</t>
+          <t>IG / TikTok</t>
         </is>
       </c>
       <c r="D13" s="12" t="inlineStr">
         <is>
-          <t>16.7k</t>
+          <t>12.4k</t>
         </is>
       </c>
       <c r="E13" s="11" t="inlineStr">
         <is>
-          <t>Collabstr (motherhood)</t>
+          <t>Collabstr (mommy)</t>
         </is>
       </c>
       <c r="F13" s="11" t="inlineStr">
         <is>
-          <t>Family / Disney / UGC</t>
+          <t>Mommy / lifestyle</t>
         </is>
       </c>
       <c r="G13" s="12" t="inlineStr">
@@ -1420,12 +1420,12 @@
       </c>
       <c r="H13" s="12" t="inlineStr">
         <is>
-          <t>2.0%</t>
+          <t>0.4% IG</t>
         </is>
       </c>
       <c r="I13" s="11" t="inlineStr">
         <is>
-          <t>$75 story / $225 3-feed</t>
+          <t>$100 feed</t>
         </is>
       </c>
       <c r="J13" s="13" t="n">
@@ -1448,19 +1448,19 @@
       </c>
       <c r="N13" s="11" t="inlineStr">
         <is>
-          <t>85% US, 85% F, 65% target age, 5.0 rating. Twentynine Palms CA. Clean family fit, fair pricing.</t>
+          <t>85% US, 96% F (highest), 68% target age. IG engagement low (0.4%) but TikTok viral (318k avg views). San Diego CA. Strong demo; value buy.</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="11" t="inlineStr">
         <is>
-          <t>Audrey Murray</t>
+          <t>Alexandra 'Jax' Molieri</t>
         </is>
       </c>
       <c r="B14" s="11" t="inlineStr">
         <is>
-          <t>@audreyinwanderlust_</t>
+          <t>@jaxdisneyfam</t>
         </is>
       </c>
       <c r="C14" s="12" t="inlineStr">
@@ -1470,7 +1470,7 @@
       </c>
       <c r="D14" s="12" t="inlineStr">
         <is>
-          <t>27.2k</t>
+          <t>16.7k</t>
         </is>
       </c>
       <c r="E14" s="11" t="inlineStr">
@@ -1480,22 +1480,22 @@
       </c>
       <c r="F14" s="11" t="inlineStr">
         <is>
-          <t>Lifestyle / motherhood</t>
+          <t>Family / Disney / UGC</t>
         </is>
       </c>
       <c r="G14" s="12" t="inlineStr">
         <is>
-          <t>66%</t>
+          <t>85%</t>
         </is>
       </c>
       <c r="H14" s="12" t="inlineStr">
         <is>
-          <t>16.3%</t>
+          <t>2.0%</t>
         </is>
       </c>
       <c r="I14" s="11" t="inlineStr">
         <is>
-          <t>$400 feed (premium)</t>
+          <t>$75 story / $225 3-feed</t>
         </is>
       </c>
       <c r="J14" s="13" t="n">
@@ -1518,54 +1518,54 @@
       </c>
       <c r="N14" s="11" t="inlineStr">
         <is>
-          <t>Very high engagement (16.3%), 83% F, 66% target age, 4.9 rating. US only 66% and pricing is premium ($375 story / $400 feed / $750 reel). Clayton NC. Strong but expensive.</t>
+          <t>85% US, 85% F, 65% target age, 5.0 rating. Twentynine Palms CA. Clean family fit, fair pricing.</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="11" t="inlineStr">
         <is>
-          <t>Keeping Up With The Griffins</t>
+          <t>Audrey Murray</t>
         </is>
       </c>
       <c r="B15" s="11" t="inlineStr">
         <is>
-          <t>(Collabstr)</t>
+          <t>@audreyinwanderlust_</t>
         </is>
       </c>
       <c r="C15" s="12" t="inlineStr">
         <is>
-          <t>IG / YouTube</t>
+          <t>IG</t>
         </is>
       </c>
       <c r="D15" s="12" t="inlineStr">
         <is>
-          <t>13.9k IG / 34.1k YT</t>
+          <t>27.2k</t>
         </is>
       </c>
       <c r="E15" s="11" t="inlineStr">
         <is>
-          <t>Collabstr (parenting)</t>
+          <t>Collabstr (motherhood)</t>
         </is>
       </c>
       <c r="F15" s="11" t="inlineStr">
         <is>
-          <t>Family / lifestyle / comedy / travel</t>
+          <t>Lifestyle / motherhood</t>
         </is>
       </c>
       <c r="G15" s="12" t="inlineStr">
         <is>
-          <t>78%</t>
+          <t>66%</t>
         </is>
       </c>
       <c r="H15" s="12" t="inlineStr">
         <is>
-          <t>1.7%</t>
+          <t>16.3%</t>
         </is>
       </c>
       <c r="I15" s="11" t="inlineStr">
         <is>
-          <t>$200 feed</t>
+          <t>$400 feed (premium)</t>
         </is>
       </c>
       <c r="J15" s="13" t="n">
@@ -1588,58 +1588,58 @@
       </c>
       <c r="N15" s="11" t="inlineStr">
         <is>
-          <t>Most-proven on the list: 5.0 rating, 13 reviews, Top Creator, Responds Fast. 78% US, 66% F, age 25-34 47%. Charleston SC. Lower engagement but the track record de-risks it.</t>
+          <t>Very high engagement (16.3%), 83% F, 66% target age, 4.9 rating. US only 66% and pricing is premium ($375 story / $400 feed / $750 reel). Clayton NC. Strong but expensive.</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="11" t="inlineStr">
         <is>
-          <t>Kaci Costello</t>
+          <t>Keeping Up With The Griffins</t>
         </is>
       </c>
       <c r="B16" s="11" t="inlineStr">
         <is>
-          <t>@kieran.and.mama</t>
+          <t>(Collabstr)</t>
         </is>
       </c>
       <c r="C16" s="12" t="inlineStr">
         <is>
-          <t>IG</t>
+          <t>IG / YouTube</t>
         </is>
       </c>
       <c r="D16" s="12" t="inlineStr">
         <is>
-          <t>18.1k</t>
+          <t>13.9k IG / 34.1k YT</t>
         </is>
       </c>
       <c r="E16" s="11" t="inlineStr">
         <is>
-          <t>Collabstr (mommy)</t>
+          <t>Collabstr (parenting)</t>
         </is>
       </c>
       <c r="F16" s="11" t="inlineStr">
         <is>
-          <t>Mommy blogger</t>
+          <t>Family / lifestyle / comedy / travel</t>
         </is>
       </c>
       <c r="G16" s="12" t="inlineStr">
         <is>
-          <t>54%</t>
+          <t>78%</t>
         </is>
       </c>
       <c r="H16" s="12" t="inlineStr">
         <is>
-          <t>n/a</t>
+          <t>1.7%</t>
         </is>
       </c>
       <c r="I16" s="11" t="inlineStr">
         <is>
-          <t>$100 feed</t>
+          <t>$200 feed</t>
         </is>
       </c>
       <c r="J16" s="13" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="K16" s="12" t="inlineStr">
         <is>
@@ -1658,19 +1658,19 @@
       </c>
       <c r="N16" s="11" t="inlineStr">
         <is>
-          <t>Budget-friendly ($100 feed / $50 story), 71% F, 66% target age. US only 54% (under our 60% floor) — flagged by the US-first screen. Hopewell Junction NY.</t>
+          <t>Most-proven on the list: 5.0 rating, 13 reviews, Top Creator, Responds Fast. 78% US, 66% F, age 25-34 47%. Charleston SC. Lower engagement but the track record de-risks it.</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="11" t="inlineStr">
         <is>
-          <t>Diana Capitao</t>
+          <t>Kaci Costello</t>
         </is>
       </c>
       <c r="B17" s="11" t="inlineStr">
         <is>
-          <t>@capitao.diana</t>
+          <t>@kieran.and.mama</t>
         </is>
       </c>
       <c r="C17" s="12" t="inlineStr">
@@ -1680,32 +1680,32 @@
       </c>
       <c r="D17" s="12" t="inlineStr">
         <is>
-          <t>14.3k</t>
+          <t>18.1k</t>
         </is>
       </c>
       <c r="E17" s="11" t="inlineStr">
         <is>
-          <t>Collabstr (parenting)</t>
+          <t>Collabstr (mommy)</t>
         </is>
       </c>
       <c r="F17" s="11" t="inlineStr">
         <is>
-          <t>Parenting expert</t>
+          <t>Mommy blogger</t>
         </is>
       </c>
       <c r="G17" s="12" t="inlineStr">
         <is>
-          <t>56%</t>
+          <t>54%</t>
         </is>
       </c>
       <c r="H17" s="12" t="inlineStr">
         <is>
-          <t>0.7%</t>
+          <t>n/a</t>
         </is>
       </c>
       <c r="I17" s="11" t="inlineStr">
         <is>
-          <t>$175 for 3 feed</t>
+          <t>$100 feed</t>
         </is>
       </c>
       <c r="J17" s="13" t="n">
@@ -1728,19 +1728,19 @@
       </c>
       <c r="N17" s="11" t="inlineStr">
         <is>
-          <t>93% F (excellent), 63% target age, best $/post ($175 for 3). US only 56% (under floor) + low engagement (0.7%). Beverly MA.</t>
+          <t>Budget-friendly ($100 feed / $50 story), 71% F, 66% target age. US only 54% (under our 60% floor) — flagged by the US-first screen. Hopewell Junction NY.</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="11" t="inlineStr">
         <is>
-          <t>Shelly Ray</t>
+          <t>Diana Capitao</t>
         </is>
       </c>
       <c r="B18" s="11" t="inlineStr">
         <is>
-          <t>@shellyraycreates</t>
+          <t>@capitao.diana</t>
         </is>
       </c>
       <c r="C18" s="12" t="inlineStr">
@@ -1750,32 +1750,32 @@
       </c>
       <c r="D18" s="12" t="inlineStr">
         <is>
-          <t>47.5k</t>
+          <t>14.3k</t>
         </is>
       </c>
       <c r="E18" s="11" t="inlineStr">
         <is>
-          <t>Collabstr (family)</t>
+          <t>Collabstr (parenting)</t>
         </is>
       </c>
       <c r="F18" s="11" t="inlineStr">
         <is>
-          <t>Family / lifestyle</t>
+          <t>Parenting expert</t>
         </is>
       </c>
       <c r="G18" s="12" t="inlineStr">
         <is>
-          <t>61%</t>
+          <t>56%</t>
         </is>
       </c>
       <c r="H18" s="12" t="inlineStr">
         <is>
-          <t>1.0%</t>
+          <t>0.7%</t>
         </is>
       </c>
       <c r="I18" s="11" t="inlineStr">
         <is>
-          <t>$450 feed (premium)</t>
+          <t>$175 for 3 feed</t>
         </is>
       </c>
       <c r="J18" s="13" t="n">
@@ -1798,12 +1798,82 @@
       </c>
       <c r="N18" s="11" t="inlineStr">
         <is>
+          <t>93% F (excellent), 63% target age, best $/post ($175 for 3). US only 56% (under floor) + low engagement (0.7%). Beverly MA.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="11" t="inlineStr">
+        <is>
+          <t>Shelly Ray</t>
+        </is>
+      </c>
+      <c r="B19" s="11" t="inlineStr">
+        <is>
+          <t>@shellyraycreates</t>
+        </is>
+      </c>
+      <c r="C19" s="12" t="inlineStr">
+        <is>
+          <t>IG</t>
+        </is>
+      </c>
+      <c r="D19" s="12" t="inlineStr">
+        <is>
+          <t>47.5k</t>
+        </is>
+      </c>
+      <c r="E19" s="11" t="inlineStr">
+        <is>
+          <t>Collabstr (family)</t>
+        </is>
+      </c>
+      <c r="F19" s="11" t="inlineStr">
+        <is>
+          <t>Family / lifestyle</t>
+        </is>
+      </c>
+      <c r="G19" s="12" t="inlineStr">
+        <is>
+          <t>61%</t>
+        </is>
+      </c>
+      <c r="H19" s="12" t="inlineStr">
+        <is>
+          <t>1.0%</t>
+        </is>
+      </c>
+      <c r="I19" s="11" t="inlineStr">
+        <is>
+          <t>$450 feed (premium)</t>
+        </is>
+      </c>
+      <c r="J19" s="13" t="n">
+        <v>3</v>
+      </c>
+      <c r="K19" s="12" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="L19" s="12" t="inlineStr">
+        <is>
+          <t>prospect</t>
+        </is>
+      </c>
+      <c r="M19" s="12" t="inlineStr">
+        <is>
+          <t>2026-06-10 (researched)</t>
+        </is>
+      </c>
+      <c r="N19" s="11" t="inlineStr">
+        <is>
           <t>Biggest following on the shortlist; 91% F, 67% target age, Top Creator, 5.0. US 61% (borderline), low engagement (1.0%), premium price ($450 feed / $650 reel). Opportunistic only.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:N18"/>
+  <autoFilter ref="A1:N19"/>
   <printOptions gridLines="1"/>
   <pageMargins left="0.3" right="0.3" top="0.5" bottom="0.5" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>

</xml_diff>